<commit_message>
Update project documentation and comments
</commit_message>
<xml_diff>
--- a/DOC/機能一覧_壁紙積算システム.xlsx
+++ b/DOC/機能一覧_壁紙積算システム.xlsx
@@ -2998,26 +2998,26 @@
       <c r="V16" s="96" t="n"/>
     </row>
     <row r="17" ht="11.25" customHeight="1" s="85">
-      <c r="A17" s="97" t="n"/>
-      <c r="B17" s="98" t="n"/>
+      <c r="A17" s="97" t="inlineStr"/>
+      <c r="B17" s="98" t="inlineStr"/>
       <c r="C17" s="89" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D17" s="88" t="inlineStr">
         <is>
-          <t>図面ページ指定機能</t>
-        </is>
-      </c>
-      <c r="E17" s="90" t="n"/>
+          <t>表ページ指定機能</t>
+        </is>
+      </c>
+      <c r="E17" s="90" t="inlineStr"/>
       <c r="F17" s="91" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G17" s="92" t="n"/>
-      <c r="H17" s="93" t="n"/>
-      <c r="I17" s="93" t="n"/>
-      <c r="J17" s="93" t="n"/>
+      <c r="G17" s="92" t="inlineStr"/>
+      <c r="H17" s="93" t="inlineStr"/>
+      <c r="I17" s="93" t="inlineStr"/>
+      <c r="J17" s="93" t="inlineStr"/>
       <c r="K17" s="93" t="n"/>
       <c r="L17" s="93" t="n"/>
       <c r="M17" s="93" t="n"/>
@@ -3338,34 +3338,26 @@
       <c r="V26" s="96" t="n"/>
     </row>
     <row r="27" ht="11.25" customHeight="1" s="85">
-      <c r="A27" s="97" t="n"/>
-      <c r="B27" s="98" t="n"/>
+      <c r="A27" s="97" t="inlineStr"/>
+      <c r="B27" s="98" t="inlineStr"/>
       <c r="C27" s="89" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D27" s="88" t="inlineStr">
         <is>
-          <t>壁紙別集計表示機能</t>
-        </is>
-      </c>
-      <c r="E27" s="90" t="n"/>
+          <t>解析状態・計算時間表示機能</t>
+        </is>
+      </c>
+      <c r="E27" s="90" t="inlineStr"/>
       <c r="F27" s="91" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="G27" s="92" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="H27" s="93" t="n"/>
-      <c r="I27" s="93" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="J27" s="93" t="n"/>
+      <c r="G27" s="92" t="inlineStr"/>
+      <c r="H27" s="93" t="inlineStr"/>
+      <c r="I27" s="93" t="inlineStr"/>
+      <c r="J27" s="93" t="inlineStr"/>
       <c r="K27" s="93" t="n"/>
       <c r="L27" s="93" t="n"/>
       <c r="M27" s="93" t="n"/>
@@ -3380,30 +3372,26 @@
       <c r="V27" s="96" t="n"/>
     </row>
     <row r="28" ht="11.25" customHeight="1" s="85">
-      <c r="A28" s="97" t="n"/>
-      <c r="B28" s="98" t="n"/>
+      <c r="A28" s="97" t="inlineStr"/>
+      <c r="B28" s="98" t="inlineStr"/>
       <c r="C28" s="89" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D28" s="88" t="inlineStr">
         <is>
-          <t>見積方式切替表示機能</t>
-        </is>
-      </c>
-      <c r="E28" s="90" t="n"/>
-      <c r="F28" s="91" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
+          <t>抽出失敗部屋警告表示機能</t>
+        </is>
+      </c>
+      <c r="E28" s="90" t="inlineStr"/>
+      <c r="F28" s="91" t="inlineStr"/>
       <c r="G28" s="92" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="H28" s="93" t="n"/>
-      <c r="I28" s="93" t="n"/>
-      <c r="J28" s="93" t="n"/>
+      <c r="H28" s="93" t="inlineStr"/>
+      <c r="I28" s="93" t="inlineStr"/>
+      <c r="J28" s="93" t="inlineStr"/>
       <c r="K28" s="93" t="n"/>
       <c r="L28" s="93" t="n"/>
       <c r="M28" s="93" t="n"/>
@@ -3690,30 +3678,30 @@
       <c r="V36" s="96" t="n"/>
     </row>
     <row r="37" ht="11.25" customHeight="1" s="85">
-      <c r="A37" s="97" t="n"/>
-      <c r="B37" s="98" t="n"/>
+      <c r="A37" s="97" t="inlineStr"/>
+      <c r="B37" s="98" t="inlineStr"/>
       <c r="C37" s="89" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D37" s="88" t="inlineStr">
         <is>
-          <t>面別壁紙選択保存機能</t>
-        </is>
-      </c>
-      <c r="E37" s="90" t="n"/>
-      <c r="F37" s="91" t="n"/>
+          <t>手動部屋追加保存機能</t>
+        </is>
+      </c>
+      <c r="E37" s="90" t="inlineStr"/>
+      <c r="F37" s="91" t="inlineStr"/>
       <c r="G37" s="92" t="inlineStr">
         <is>
-          <t>U</t>
-        </is>
-      </c>
-      <c r="H37" s="93" t="n"/>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H37" s="93" t="inlineStr"/>
       <c r="I37" s="93" t="inlineStr">
         <is>
           <t>R</t>
         </is>
       </c>
-      <c r="J37" s="93" t="n"/>
+      <c r="J37" s="93" t="inlineStr"/>
       <c r="K37" s="93" t="n"/>
       <c r="L37" s="93" t="n"/>
       <c r="M37" s="93" t="n"/>
@@ -3728,26 +3716,26 @@
       <c r="V37" s="96" t="n"/>
     </row>
     <row r="38" ht="11.25" customHeight="1" s="85">
-      <c r="A38" s="97" t="n"/>
-      <c r="B38" s="98" t="n"/>
+      <c r="A38" s="97" t="inlineStr"/>
+      <c r="B38" s="98" t="inlineStr"/>
       <c r="C38" s="89" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D38" s="88" t="inlineStr">
         <is>
-          <t>面別面積・開口部保存機能</t>
-        </is>
-      </c>
-      <c r="E38" s="90" t="n"/>
-      <c r="F38" s="91" t="n"/>
+          <t>集計対象外設定保存機能</t>
+        </is>
+      </c>
+      <c r="E38" s="90" t="inlineStr"/>
+      <c r="F38" s="91" t="inlineStr"/>
       <c r="G38" s="92" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="H38" s="93" t="n"/>
-      <c r="I38" s="93" t="n"/>
-      <c r="J38" s="93" t="n"/>
+      <c r="H38" s="93" t="inlineStr"/>
+      <c r="I38" s="93" t="inlineStr"/>
+      <c r="J38" s="93" t="inlineStr"/>
       <c r="K38" s="93" t="n"/>
       <c r="L38" s="93" t="n"/>
       <c r="M38" s="93" t="n"/>
@@ -3950,26 +3938,26 @@
       <c r="V44" s="96" t="n"/>
     </row>
     <row r="45" ht="11.25" customHeight="1" s="85">
-      <c r="A45" s="97" t="n"/>
-      <c r="B45" s="98" t="n"/>
+      <c r="A45" s="97" t="inlineStr"/>
+      <c r="B45" s="98" t="inlineStr"/>
       <c r="C45" s="89" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D45" s="88" t="inlineStr">
         <is>
-          <t>既存部屋置換機能</t>
-        </is>
-      </c>
-      <c r="E45" s="90" t="n"/>
-      <c r="F45" s="91" t="n"/>
-      <c r="G45" s="92" t="inlineStr">
-        <is>
-          <t>CD</t>
-        </is>
-      </c>
-      <c r="H45" s="93" t="n"/>
-      <c r="I45" s="93" t="n"/>
-      <c r="J45" s="93" t="n"/>
+          <t>PDF解析状態更新機能</t>
+        </is>
+      </c>
+      <c r="E45" s="90" t="inlineStr"/>
+      <c r="F45" s="91" t="inlineStr">
+        <is>
+          <t>U</t>
+        </is>
+      </c>
+      <c r="G45" s="92" t="inlineStr"/>
+      <c r="H45" s="93" t="inlineStr"/>
+      <c r="I45" s="93" t="inlineStr"/>
+      <c r="J45" s="93" t="inlineStr"/>
       <c r="K45" s="93" t="n"/>
       <c r="L45" s="93" t="n"/>
       <c r="M45" s="93" t="n"/>

</xml_diff>